<commit_message>
Reconcile SYSCTRL schedules and select Molex NFC antenna
</commit_message>
<xml_diff>
--- a/SYS/ADHERENT_System_Diagram_Components_R27.xlsx
+++ b/SYS/ADHERENT_System_Diagram_Components_R27.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="1" r:id="Rce178e0695d6442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="R5565c59938eb411e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="1" r:id="Ra60fc5e173794ff1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="Rf5dcb6ee9c84404b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -73,7 +73,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -108,6 +108,9 @@
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -116,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DiagramComponents" displayName="DiagramComponents" ref="A6:J80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DiagramComponents" displayName="DiagramComponents" ref="A6:J88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Ref"/>
     <x:tableColumn id="2" name="Diagram block / location"/>
@@ -368,7 +371,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="1" t="str">
-        <x:v>Source: Electrical_System_Level_Wiring_Diagram_R27.drawio. Quantities per machine; junction boxes are removed. TBC = not yet confirmed.</x:v>
+        <x:v>Current SYSCTRL topology: onboard SMPS and power connectors; no independent distribution unit. NFC antenna selected: Molex 1462362151.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -530,7 +533,7 @@
         <x:v>SELECTED / engineering pending</x:v>
       </x:c>
       <x:c r="I9" s="4" t="str">
-        <x:v>Buck and drivers pending; local servo rail voltage TBC.</x:v>
+        <x:v>Single 24 V system input; integrated power routing/connectors and one 12 V SMPS. Protection and local servo rail pending.</x:v>
       </x:c>
       <x:c r="J9" s="4" t="str">
         <x:v>S01/S03/S04</x:v>
@@ -669,28 +672,28 @@
         <x:v>DIST24</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>24 V distribution</x:v>
+        <x:v>SYSCTRL power connectors / internal routing</x:v>
       </x:c>
       <x:c r="C14" s="7" t="str">
-        <x:v>24 V main distribution and terminals</x:v>
+        <x:v>SYSCTRL 24 V distribution function</x:v>
       </x:c>
       <x:c r="D14" s="7" t="str">
         <x:v>TBC</x:v>
       </x:c>
       <x:c r="E14" s="7" t="str">
-        <x:v>TBC</x:v>
+        <x:v>Internal PCB routing / connectors; MPN TBC</x:v>
       </x:c>
       <x:c r="F14" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G14" s="7" t="str">
-        <x:v>BUY</x:v>
+        <x:v>IN SYSCTRL</x:v>
       </x:c>
       <x:c r="H14" s="7" t="str">
-        <x:v>HOLD</x:v>
+        <x:v>INTERNAL / HOLD</x:v>
       </x:c>
       <x:c r="I14" s="7" t="str">
-        <x:v>Must carry total PSU output; not one 6.3 A fuse holder.</x:v>
+        <x:v>Functional allocation within SYSCTRL; not an independent distribution assembly. Do not buy as a separate module.</x:v>
       </x:c>
       <x:c r="J14" s="7" t="str">
         <x:v>O06</x:v>
@@ -701,28 +704,28 @@
         <x:v>DIST12</x:v>
       </x:c>
       <x:c r="B15" s="4" t="str">
-        <x:v>12 V distribution</x:v>
+        <x:v>SYSCTRL power connectors / internal routing</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
-        <x:v>Separate derived 12 V distribution</x:v>
+        <x:v>SYSCTRL derived 12 V distribution function</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
         <x:v>TBC</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
-        <x:v>TBC</x:v>
+        <x:v>Internal PCB routing / connectors; MPN TBC</x:v>
       </x:c>
       <x:c r="F15" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="4" t="str">
-        <x:v>BUY</x:v>
+        <x:v>IN SYSCTRL</x:v>
       </x:c>
       <x:c r="H15" s="4" t="str">
-        <x:v>HOLD</x:v>
+        <x:v>INTERNAL / HOLD</x:v>
       </x:c>
       <x:c r="I15" s="4" t="str">
-        <x:v>Fed from SYSCTRL J43/W04.</x:v>
+        <x:v>Functional allocation within SYSCTRL; not an independent distribution assembly. Do not buy as a separate module.</x:v>
       </x:c>
       <x:c r="J15" s="4" t="str">
         <x:v>O02/O06</x:v>
@@ -733,28 +736,28 @@
         <x:v>DIN-F</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>F1-F13, F15-F18</x:v>
+        <x:v>Withdrawn DIN-holder allocation</x:v>
       </x:c>
       <x:c r="C16" s="7" t="str">
-        <x:v>DIN fuse positions</x:v>
+        <x:v>Previous DIN fuse-holder assumption</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
         <x:v>Phoenix Contact</x:v>
       </x:c>
       <x:c r="E16" s="7" t="str">
-        <x:v>3046032 / UT 4-HESI (5X20), candidate</x:v>
+        <x:v>No released holder selection</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="7" t="str">
-        <x:v>BUY</x:v>
+        <x:v>RETIRED</x:v>
       </x:c>
       <x:c r="H16" s="7" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>WITHDRAWN</x:v>
       </x:c>
       <x:c r="I16" s="7" t="str">
-        <x:v>F1–F13 and F15–F18; F12 holder/current must be reselected if necessary.</x:v>
+        <x:v>The previous 17 x Phoenix 3046032 assumption is withdrawn. Final branch-protection implementation and physical quantities TBC.</x:v>
       </x:c>
       <x:c r="J16" s="7" t="str">
         <x:v>S11/O06</x:v>
@@ -768,25 +771,25 @@
         <x:v>F1-F18</x:v>
       </x:c>
       <x:c r="C17" s="4" t="str">
-        <x:v>Fuse elements</x:v>
+        <x:v>Branch-protection references</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
         <x:v>TBC</x:v>
       </x:c>
       <x:c r="E17" s="4" t="str">
-        <x:v>TBC by branch schedule</x:v>
+        <x:v>TBC by branch design</x:v>
       </x:c>
       <x:c r="F17" s="8" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="G17" s="4" t="str">
-        <x:v>BUY</x:v>
+        <x:v>FUNCTIONAL COUNT</x:v>
       </x:c>
       <x:c r="H17" s="4" t="str">
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="I17" s="4" t="str">
-        <x:v>17 DIN + F14 on SYSCTRL; element curves/DC interruption/ratings not released.</x:v>
+        <x:v>18 protected branch references, not 18 finalized fuse elements. Select technology, placement, ratings and actual purchase counts during SYSCTRL design.</x:v>
       </x:c>
       <x:c r="J17" s="4" t="str">
         <x:v>Fuses/O06</x:v>
@@ -800,7 +803,7 @@
         <x:v>SYSCTRL buck</x:v>
       </x:c>
       <x:c r="C18" s="7" t="str">
-        <x:v>On-board 24→12 V converter</x:v>
+        <x:v>Onboard 24 V-to-12 V SMPS</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
         <x:v>TBC</x:v>
@@ -818,7 +821,7 @@
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="I18" s="7" t="str">
-        <x:v>Not a separate module; include in SYSCTRL component BOM when designed.</x:v>
+        <x:v>One conversion stage inside SYSCTRL. Input/output rails are internal; no external converter or distribution module.</x:v>
       </x:c>
       <x:c r="J18" s="7" t="str">
         <x:v>O02</x:v>
@@ -1661,10 +1664,10 @@
         <x:v>NFC</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
-        <x:v>Optional NFC / card</x:v>
+        <x:v>NFC front end; board allocation TBC</x:v>
       </x:c>
       <x:c r="C45" s="4" t="str">
-        <x:v>NFC/payment reader</x:v>
+        <x:v>NFC reader / front-end function</x:v>
       </x:c>
       <x:c r="D45" s="4" t="str">
         <x:v>TBC</x:v>
@@ -1673,19 +1676,19 @@
         <x:v>TBC</x:v>
       </x:c>
       <x:c r="F45" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G45" s="4" t="str">
-        <x:v>OPTION</x:v>
+        <x:v>FUNCTIONAL ALLOWANCE</x:v>
       </x:c>
       <x:c r="H45" s="4" t="str">
-        <x:v>EXCLUDED</x:v>
+        <x:v>HOLD O16</x:v>
       </x:c>
       <x:c r="I45" s="4" t="str">
-        <x:v>Not approved; excluded from committed quantities and power subtotal.</x:v>
+        <x:v>One reader function planned for selected antenna; IC/module, board allocation, host interface, supply and implementation quantity pending. Not a selected payment terminal.</x:v>
       </x:c>
       <x:c r="J45" s="4" t="str">
-        <x:v>O13</x:v>
+        <x:v>O16</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="46" customHeight="1">
@@ -2182,7 +2185,7 @@
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E61" s="4" t="str">
-        <x:v>TBC - native terminal / mating part</x:v>
+        <x:v>–</x:v>
       </x:c>
       <x:c r="F61" s="8" t="n">
         <x:v>2</x:v>
@@ -2461,28 +2464,28 @@
         <x:v>IF-J29</x:v>
       </x:c>
       <x:c r="B70" s="7" t="str">
-        <x:v>SYSCTRL</x:v>
+        <x:v>SYSCTRL internal function</x:v>
       </x:c>
       <x:c r="C70" s="7" t="str">
-        <x:v>24 V motor supply in (F11)</x:v>
+        <x:v>Former external motor-rail input W06</x:v>
       </x:c>
       <x:c r="D70" s="7" t="str">
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E70" s="7" t="str">
-        <x:v>TBC</x:v>
+        <x:v>Not fitted for former loop</x:v>
       </x:c>
       <x:c r="F70" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G70" s="7" t="str">
         <x:v>INTERFACE POSITIONS</x:v>
       </x:c>
       <x:c r="H70" s="7" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>RETIRED ALLOCATION</x:v>
       </x:c>
       <x:c r="I70" s="7" t="str">
-        <x:v>Power connector; pin count/gauge/current TBC. Mate: TBC. Final mating set, keying, gauge and derating require approval.</x:v>
+        <x:v>No external connector assigned. Mate: Not fitted. Legacy reference retained; no extra external cable/mate. Final SYSCTRL connector references below remain TBC.</x:v>
       </x:c>
       <x:c r="J70" s="7" t="str">
         <x:v>Electrical workbook / Connectors</x:v>
@@ -2502,7 +2505,7 @@
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E71" s="4" t="str">
-        <x:v>TBC - native terminal / mating part</x:v>
+        <x:v>ferrule</x:v>
       </x:c>
       <x:c r="F71" s="8" t="n">
         <x:v>4</x:v>
@@ -2534,7 +2537,7 @@
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E72" s="7" t="str">
-        <x:v>TBC - native terminal / mating part</x:v>
+        <x:v>ferrule</x:v>
       </x:c>
       <x:c r="F72" s="9" t="n">
         <x:v>5</x:v>
@@ -2557,28 +2560,28 @@
         <x:v>IF-J41</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
-        <x:v>SYSCTRL</x:v>
+        <x:v>SYSCTRL internal function</x:v>
       </x:c>
       <x:c r="C73" s="4" t="str">
-        <x:v>24 V input from F12 to on-board buck</x:v>
+        <x:v>Former external SMPS input W07</x:v>
       </x:c>
       <x:c r="D73" s="4" t="str">
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E73" s="4" t="str">
-        <x:v>TBC</x:v>
+        <x:v>Not fitted for former loop</x:v>
       </x:c>
       <x:c r="F73" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G73" s="4" t="str">
         <x:v>INTERFACE POSITIONS</x:v>
       </x:c>
       <x:c r="H73" s="4" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>RETIRED ALLOCATION</x:v>
       </x:c>
       <x:c r="I73" s="4" t="str">
-        <x:v>Power connector; input current TBC. Mate: TBC. Final mating set, keying, gauge and derating require approval.</x:v>
+        <x:v>No external connector assigned. Mate: Not fitted. Legacy reference retained; no extra external cable/mate. Final SYSCTRL connector references below remain TBC.</x:v>
       </x:c>
       <x:c r="J73" s="4" t="str">
         <x:v>Electrical workbook / Connectors</x:v>
@@ -2630,7 +2633,7 @@
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E75" s="4" t="str">
-        <x:v>TBC - native terminal / mating part</x:v>
+        <x:v>–</x:v>
       </x:c>
       <x:c r="F75" s="8" t="n">
         <x:v>1</x:v>
@@ -2694,7 +2697,7 @@
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E77" s="4" t="str">
-        <x:v>TBC - native terminal / mating part</x:v>
+        <x:v>ferrule</x:v>
       </x:c>
       <x:c r="F77" s="8" t="n">
         <x:v>1</x:v>
@@ -2717,28 +2720,28 @@
         <x:v>IF-J43</x:v>
       </x:c>
       <x:c r="B78" s="7" t="str">
-        <x:v>SYSCTRL</x:v>
+        <x:v>SYSCTRL internal function</x:v>
       </x:c>
       <x:c r="C78" s="7" t="str">
-        <x:v>12 V buck output to distribution</x:v>
+        <x:v>Former external SMPS output loop W04</x:v>
       </x:c>
       <x:c r="D78" s="7" t="str">
         <x:v>Native / TBC</x:v>
       </x:c>
       <x:c r="E78" s="7" t="str">
-        <x:v>TBC</x:v>
+        <x:v>Not fitted for former loop</x:v>
       </x:c>
       <x:c r="F78" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G78" s="7" t="str">
         <x:v>INTERFACE POSITIONS</x:v>
       </x:c>
       <x:c r="H78" s="7" t="str">
-        <x:v>HOLD O02</x:v>
+        <x:v>RETIRED ALLOCATION</x:v>
       </x:c>
       <x:c r="I78" s="7" t="str">
-        <x:v>Power connector; output current TBC. Mate: TBC. W04; not an external 12 V input.</x:v>
+        <x:v>No external connector assigned. Mate: Not fitted. Legacy reference retained; no extra external cable/mate. Final SYSCTRL connector references below remain TBC.</x:v>
       </x:c>
       <x:c r="J78" s="7" t="str">
         <x:v>Electrical workbook / Connectors</x:v>
@@ -2803,6 +2806,262 @@
         <x:v>Bonding lugs and PE terminals. Mate: TBC. W37 bonding assembly; counts await enclosure bonding plan.</x:v>
       </x:c>
       <x:c r="J80" s="7" t="str">
+        <x:v>Electrical workbook / Connectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="46" customHeight="1">
+      <x:c r="A81" s="4" t="str">
+        <x:v>ANT-NFC</x:v>
+      </x:c>
+      <x:c r="B81" s="4" t="str">
+        <x:v>NFC antenna</x:v>
+      </x:c>
+      <x:c r="C81" s="4" t="str">
+        <x:v>NFC antenna</x:v>
+      </x:c>
+      <x:c r="D81" s="4" t="str">
+        <x:v>Molex</x:v>
+      </x:c>
+      <x:c r="E81" s="4" t="str">
+        <x:v>1462362151</x:v>
+      </x:c>
+      <x:c r="F81" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G81" s="4" t="str">
+        <x:v>BUY</x:v>
+      </x:c>
+      <x:c r="H81" s="4" t="str">
+        <x:v>SELECTED / integration pending</x:v>
+      </x:c>
+      <x:c r="I81" s="4" t="str">
+        <x:v>13.56 MHz; 15 x 15 x 0.27 mm; adhesive; 102 mm cable; 2.40 uH. One per machine planning quantity. Reader matching, termination and mounting TBC.</x:v>
+      </x:c>
+      <x:c r="J81" s="4" t="str">
+        <x:v>S14/S15/O16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="46" customHeight="1">
+      <x:c r="A82" s="4" t="str">
+        <x:v>IF-SYSCTRL-PWR-IN (TBC)</x:v>
+      </x:c>
+      <x:c r="B82" s="4" t="str">
+        <x:v>SYSCTRL</x:v>
+      </x:c>
+      <x:c r="C82" s="4" t="str">
+        <x:v>24 V system power input</x:v>
+      </x:c>
+      <x:c r="D82" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="E82" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="F82" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G82" s="4" t="str">
+        <x:v>INTERFACE POSITIONS</x:v>
+      </x:c>
+      <x:c r="H82" s="4" t="str">
+        <x:v>HOLD O06</x:v>
+      </x:c>
+      <x:c r="I82" s="4" t="str">
+        <x:v>Power connector rated for total machine input; TBC. Mate: PSU1 screw terminals to selected SYSCTRL mate. W03. Rating, gauge, inrush and PCB current paths must cover all simultaneous loads.</x:v>
+      </x:c>
+      <x:c r="J82" s="4" t="str">
+        <x:v>Electrical workbook / Connectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="46" customHeight="1">
+      <x:c r="A83" s="4" t="str">
+        <x:v>IF-SYSCTRL-24V-LANE (TBC)</x:v>
+      </x:c>
+      <x:c r="B83" s="4" t="str">
+        <x:v>SYSCTRL</x:v>
+      </x:c>
+      <x:c r="C83" s="4" t="str">
+        <x:v>24 V row power outputs</x:v>
+      </x:c>
+      <x:c r="D83" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="E83" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="F83" s="4" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G83" s="4" t="str">
+        <x:v>INTERFACE POSITIONS</x:v>
+      </x:c>
+      <x:c r="H83" s="4" t="str">
+        <x:v>HOLD O06</x:v>
+      </x:c>
+      <x:c r="I83" s="4" t="str">
+        <x:v>F1-F10 branch outputs; connector MPN/pins TBC. Mate: LANECTRL J5 candidate. W24, ten branch circuits. Physical housings may combine circuits; packaging TBC.</x:v>
+      </x:c>
+      <x:c r="J83" s="4" t="str">
+        <x:v>Electrical workbook / Connectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="46" customHeight="1">
+      <x:c r="A84" s="4" t="str">
+        <x:v>IF-SYSCTRL-24V-DRIVE (TBC)</x:v>
+      </x:c>
+      <x:c r="B84" s="4" t="str">
+        <x:v>SYSCTRL</x:v>
+      </x:c>
+      <x:c r="C84" s="4" t="str">
+        <x:v>Proposed 24 V X/Z drive outputs</x:v>
+      </x:c>
+      <x:c r="D84" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="E84" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="F84" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G84" s="4" t="str">
+        <x:v>INTERFACE POSITIONS</x:v>
+      </x:c>
+      <x:c r="H84" s="4" t="str">
+        <x:v>HOLD O01/O06</x:v>
+      </x:c>
+      <x:c r="I84" s="4" t="str">
+        <x:v>F15/F16 branch outputs; connector MPN/pins TBC. Mate: Native drive mates TBC. W29/W30. 24 V compatibility and current need supplier evidence.</x:v>
+      </x:c>
+      <x:c r="J84" s="4" t="str">
+        <x:v>Electrical workbook / Connectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="46" customHeight="1">
+      <x:c r="A85" s="4" t="str">
+        <x:v>IF-SYSCTRL-24V-IO (TBC)</x:v>
+      </x:c>
+      <x:c r="B85" s="4" t="str">
+        <x:v>SYSCTRL</x:v>
+      </x:c>
+      <x:c r="C85" s="4" t="str">
+        <x:v>24 V IOCTRL module output</x:v>
+      </x:c>
+      <x:c r="D85" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="E85" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="F85" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G85" s="4" t="str">
+        <x:v>INTERFACE POSITIONS</x:v>
+      </x:c>
+      <x:c r="H85" s="4" t="str">
+        <x:v>HOLD O06</x:v>
+      </x:c>
+      <x:c r="I85" s="4" t="str">
+        <x:v>F17 branch output; connector MPN/pins TBC. Mate: IOCTRL native power terminals. W34. Separate from 12 V relay-contact feed.</x:v>
+      </x:c>
+      <x:c r="J85" s="4" t="str">
+        <x:v>Electrical workbook / Connectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="46" customHeight="1">
+      <x:c r="A86" s="4" t="str">
+        <x:v>IF-SYSCTRL-12V-MAIN (TBC)</x:v>
+      </x:c>
+      <x:c r="B86" s="4" t="str">
+        <x:v>SYSCTRL</x:v>
+      </x:c>
+      <x:c r="C86" s="4" t="str">
+        <x:v>Derived 12 V MAINCTRL output</x:v>
+      </x:c>
+      <x:c r="D86" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="E86" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="F86" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G86" s="4" t="str">
+        <x:v>INTERFACE POSITIONS</x:v>
+      </x:c>
+      <x:c r="H86" s="4" t="str">
+        <x:v>HOLD O02/O06</x:v>
+      </x:c>
+      <x:c r="I86" s="4" t="str">
+        <x:v>F13 branch output; connector MPN/pins TBC. Mate: MYIR J46 native power plug TBC. W05. Generated by the single onboard SMPS.</x:v>
+      </x:c>
+      <x:c r="J86" s="4" t="str">
+        <x:v>Electrical workbook / Connectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="46" customHeight="1">
+      <x:c r="A87" s="4" t="str">
+        <x:v>IF-SYSCTRL-12V-LATCH (TBC)</x:v>
+      </x:c>
+      <x:c r="B87" s="4" t="str">
+        <x:v>SYSCTRL</x:v>
+      </x:c>
+      <x:c r="C87" s="4" t="str">
+        <x:v>Derived 12 V latch-contact output</x:v>
+      </x:c>
+      <x:c r="D87" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="E87" s="4" t="str">
+        <x:v>TBC</x:v>
+      </x:c>
+      <x:c r="F87" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G87" s="4" t="str">
+        <x:v>INTERFACE POSITIONS</x:v>
+      </x:c>
+      <x:c r="H87" s="4" t="str">
+        <x:v>HOLD O02/O06</x:v>
+      </x:c>
+      <x:c r="I87" s="4" t="str">
+        <x:v>F18 branch output; connector MPN/pins TBC. Mate: IOCTRL relay COM terminals. W35. Lane-logic 12 V is already allocated to J15A; do not duplicate it.</x:v>
+      </x:c>
+      <x:c r="J87" s="4" t="str">
+        <x:v>Electrical workbook / Connectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="55" customHeight="1">
+      <x:c r="A88" s="4" t="str">
+        <x:v>IF-NFC-RF (TBC)</x:v>
+      </x:c>
+      <x:c r="B88" s="4" t="str">
+        <x:v>Antenna / reader location TBC</x:v>
+      </x:c>
+      <x:c r="C88" s="4" t="str">
+        <x:v>NFC antenna to reader front end</x:v>
+      </x:c>
+      <x:c r="D88" s="4" t="str">
+        <x:v>Molex antenna; reader TBC</x:v>
+      </x:c>
+      <x:c r="E88" s="4" t="str">
+        <x:v>Molex 1462362151 antenna</x:v>
+      </x:c>
+      <x:c r="F88" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G88" s="4" t="str">
+        <x:v>INTERFACE POSITIONS</x:v>
+      </x:c>
+      <x:c r="H88" s="4" t="str">
+        <x:v>HOLD O16</x:v>
+      </x:c>
+      <x:c r="I88" s="4" t="str">
+        <x:v>RF termination and matching TBC. Mate: Reader-side connection TBC. 102 mm antenna cable is included in the selected antenna; not a separately selected coax jumper. Verify actual termination from drawing.</x:v>
+      </x:c>
+      <x:c r="J88" s="4" t="str">
         <x:v>Electrical workbook / Connectors</x:v>
       </x:c>
     </x:row>
@@ -2815,7 +3074,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92ef9d1e866347b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb54c86f6f7c841f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2855,7 +3114,7 @@
         <x:v>brain.md and user decisions through 2026-09-24</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
-        <x:v>Single 24 V PSU; SYSCTRL-derived 12 V; IOCTRL naming; 70 lanes; no UPS/cellular. No junction boxes; sensors connect directly to controller boards.</x:v>
+        <x:v>SYSCTRL contains power distribution/connectors and one 24 V-to-12 V SMPS. No junction boxes. NFC antenna selected; reader integration pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="55" customHeight="1">
@@ -3028,7 +3287,35 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>O01-O15: see OpenItems in APDU_Electrical_Tables_R27.xlsx. Connector part candidates are carried from that workbook.</x:v>
+        <x:v>OpenItems O01-O16: see APDU_Electrical_Tables_R27.xlsx. Quantities include internal functional allocations and interface positions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="65" customHeight="1">
+      <x:c r="A18" s="14" t="str">
+        <x:v>S14</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>Molex NFC antenna</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>https://www.molex.com/en-us/products/part-detail/1462362151</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>1462362151: 13.56 MHz, 2.40 uH; 15 x 15 x 0.27 mm, adhesive, 102 mm cable. Manufacturer specifications; integration pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="65" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>S15</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>User-selected distributor listing</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/molex/1462362151/15204370</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>User selected this antenna. Antenna selection does not select the NFC reader or payment functionality.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>